<commit_message>
Update for Magistrate queries.
</commit_message>
<xml_diff>
--- a/data/Conditions_Queries.xlsx
+++ b/data/Conditions_Queries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIS\Henrico\Henrico_Data_2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5DF2DD-5AA1-4A54-BBFA-37B7CB63FEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773DD919-EAC2-489B-A162-B5470833AF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{35C825B9-898A-46C9-A18E-DC972BBDF846}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{35C825B9-898A-46C9-A18E-DC972BBDF846}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4671,27 +4671,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed0ff079-217a-47d4-b7ec-91b316da1e03">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="3042e918-aefc-4171-9d6c-c740f3c2ff7c" xsi:nil="true"/>
-    <Status xmlns="ed0ff079-217a-47d4-b7ec-91b316da1e03" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001F1BD6F70B794D4A83A1A74C1C7FFB13" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a36ec311cb1a64ba9887f4cfe263bcf0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ed0ff079-217a-47d4-b7ec-91b316da1e03" xmlns:ns3="3042e918-aefc-4171-9d6c-c740f3c2ff7c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b5d2f1e144e455241c9e34cacdc13afb" ns2:_="" ns3:_="">
     <xsd:import namespace="ed0ff079-217a-47d4-b7ec-91b316da1e03"/>
@@ -4934,10 +4913,42 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="ed0ff079-217a-47d4-b7ec-91b316da1e03">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="3042e918-aefc-4171-9d6c-c740f3c2ff7c" xsi:nil="true"/>
+    <Status xmlns="ed0ff079-217a-47d4-b7ec-91b316da1e03" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0627FB08-4574-4A0A-A2C4-FFFB20FF76D4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2AA363C-5FFF-4389-992E-0B1456F9F257}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="ed0ff079-217a-47d4-b7ec-91b316da1e03"/>
+    <ds:schemaRef ds:uri="3042e918-aefc-4171-9d6c-c740f3c2ff7c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4960,20 +4971,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2AA363C-5FFF-4389-992E-0B1456F9F257}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0627FB08-4574-4A0A-A2C4-FFFB20FF76D4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="ed0ff079-217a-47d4-b7ec-91b316da1e03"/>
-    <ds:schemaRef ds:uri="3042e918-aefc-4171-9d6c-c740f3c2ff7c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>